<commit_message>
Working on TC Development
created the first couple test cases (not yet executed)
</commit_message>
<xml_diff>
--- a/Manual-Testing/SauceDemo/TestCases/SauceDemo_TestCases.xlsx
+++ b/Manual-Testing/SauceDemo/TestCases/SauceDemo_TestCases.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CodingProjects\QA-Portfolio\Manual-Testing\SauceDemo\TestCases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniellebuonpane/Desktop/CodingProjects/QA-Portfolio/Manual-Testing/SauceDemo/TestCases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8689538D-6DD2-437F-AB44-4A0B3B208D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCA02B79-B0A6-D047-8A0B-9B1855EB662D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-210" windowWidth="29040" windowHeight="15720" xr2:uid="{4C38DD76-CF43-4CD3-BDA5-DD01809C6AAE}"/>
+    <workbookView xWindow="20" yWindow="500" windowWidth="24640" windowHeight="15500" xr2:uid="{4C38DD76-CF43-4CD3-BDA5-DD01809C6AAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
     <sheet name="Severity &amp; Priority Key " sheetId="2" r:id="rId2"/>
+    <sheet name="TC Naming Convention" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="64">
   <si>
     <t>BRING ME BACK TO THE TEST CASES!</t>
   </si>
@@ -163,6 +163,81 @@
   </si>
   <si>
     <t>Helpful Link(s)</t>
+  </si>
+  <si>
+    <t>Select to view the Test Case Naming Convention Guildelines</t>
+  </si>
+  <si>
+    <t>Test Case ID Naming Convention Guidelines</t>
+  </si>
+  <si>
+    <t>Test Case ID's will all be structured using 4 components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Module Prefix </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Subcategory </t>
+  </si>
+  <si>
+    <t>3. Test Number (sequential)</t>
+  </si>
+  <si>
+    <t>4. Persona Indicator (for persona tests)</t>
+  </si>
+  <si>
+    <t>AUTH-LOGIN-001</t>
+  </si>
+  <si>
+    <t>AUTH-LOGIN-002-USR-LOCKED</t>
+  </si>
+  <si>
+    <t>TC ID Examples</t>
+  </si>
+  <si>
+    <t>No persona - (user story: a casual user should be able to become a registered user by logging in with valid user credentials)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Using perona - (user story: a user who is locked out of the system should not be able to login using valid credentials </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-LOGIN-001 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login with valid credentials </t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a </t>
+  </si>
+  <si>
+    <t xml:space="preserve">User authentication using standard-user persona  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. navigate to saucedemo.com
+2. enter "standard_user" to the username field 
+3. enter "secret_sauce" to the password field 
+4. click "Login" button </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(a) the user is brought to the inventory.html page (view within the page URL) 
+(b) the user can view "products" just below the "=" menu 
+(c) the cart icon is now visible in the top right of the page </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTH-LOGIN-002 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login with invalid credentials </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. navigate to saucedemo.com
+2. enter "standard_user" to the username field 
+3. enter "secret" to the password field 
+4. click "Login" button </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(a) the user does not move from the login page 
+(b) an error message displays indicating the failed login attempt </t>
   </si>
 </sst>
 </file>
@@ -172,7 +247,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mm/dd/yyyy\ h:mm\ AM/PM;@"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -236,6 +311,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -251,7 +361,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -369,6 +479,251 @@
         <color indexed="64"/>
       </left>
       <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -384,25 +739,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -420,6 +763,113 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -428,6 +878,12 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -589,12 +1045,6 @@
         <scheme val="none"/>
       </font>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -614,19 +1064,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB1DF94C-0755-4907-BE7F-A1A1E83D49A2}" name="Table1" displayName="Table1" ref="A6:J7" totalsRowShown="0" dataDxfId="10">
-  <autoFilter ref="A6:J7" xr:uid="{BB1DF94C-0755-4907-BE7F-A1A1E83D49A2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB1DF94C-0755-4907-BE7F-A1A1E83D49A2}" name="Table1" displayName="Table1" ref="A6:J9" totalsRowShown="0" dataDxfId="12">
+  <autoFilter ref="A6:J9" xr:uid="{BB1DF94C-0755-4907-BE7F-A1A1E83D49A2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{B011EBE0-F8AD-4DD8-BE71-830A8FA49270}" name="Test Case ID " dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{C47D0AD3-C0D2-4721-BFDA-48A86F3DA9E9}" name="Feature/Module" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{4F9A7D38-CBD8-4899-A573-E96697D869CD}" name="Test Scenario " dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{1454AAC5-8DFB-47ED-A2F7-C0947EC4B23D}" name="Preconditions" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{8030947D-1C87-4E6A-A4E4-8C3FA4F0C06E}" name="Test Steps " dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{7836C71F-EDA6-45DC-945C-66CBBD11898A}" name="Expected Results " dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{014D84C0-1923-4E15-BFB4-B001E4225D24}" name="Actual Results " dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{7832FEF6-B58E-492F-8F0A-ECCA519ACBCB}" name="Status (ex. Pass/Fail) " dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{5D07A50D-6F6D-4EBE-BC31-B38BC542353A}" name="Severity/Priority" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{E6A9E6E3-0AF1-412B-BA75-BE2F2542DF50}" name="Comments/Attachments" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{B011EBE0-F8AD-4DD8-BE71-830A8FA49270}" name="Test Case ID " dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{C47D0AD3-C0D2-4721-BFDA-48A86F3DA9E9}" name="Feature/Module" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{4F9A7D38-CBD8-4899-A573-E96697D869CD}" name="Test Scenario " dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{1454AAC5-8DFB-47ED-A2F7-C0947EC4B23D}" name="Preconditions" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{8030947D-1C87-4E6A-A4E4-8C3FA4F0C06E}" name="Test Steps " dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{7836C71F-EDA6-45DC-945C-66CBBD11898A}" name="Expected Results " dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{014D84C0-1923-4E15-BFB4-B001E4225D24}" name="Actual Results " dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{7832FEF6-B58E-492F-8F0A-ECCA519ACBCB}" name="Status (ex. Pass/Fail) " dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{5D07A50D-6F6D-4EBE-BC31-B38BC542353A}" name="Severity/Priority" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{E6A9E6E3-0AF1-412B-BA75-BE2F2542DF50}" name="Comments/Attachments" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -637,7 +1087,7 @@
   <autoFilter ref="A5:B9" xr:uid="{3539645C-9398-4EB9-A187-25742C885B7D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D38191A1-A192-44F7-8CC1-2049E6D6718B}" name="Value  "/>
-    <tableColumn id="2" xr3:uid="{F91F5124-E7F9-4AAB-B0C8-83D4C664F212}" name="Definition " dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{F91F5124-E7F9-4AAB-B0C8-83D4C664F212}" name="Definition " dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight3" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -648,7 +1098,7 @@
   <autoFilter ref="D5:E8" xr:uid="{D8369E32-4F2F-4C26-951E-A09F7F378591}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{AABD4610-0881-46F2-B38C-2F085F954B54}" name="Value "/>
-    <tableColumn id="2" xr3:uid="{66E9AA3F-59E8-4A4A-8D2F-4F168108B62B}" name="Definition " dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{66E9AA3F-59E8-4A4A-8D2F-4F168108B62B}" name="Definition " dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -971,67 +1421,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025E7C9E-74E3-4BF8-8479-330E9E029DCD}">
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="28.7109375" customWidth="1"/>
-    <col min="3" max="3" width="41.42578125" customWidth="1"/>
-    <col min="4" max="4" width="45.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.7109375" customWidth="1"/>
-    <col min="6" max="6" width="30.85546875" customWidth="1"/>
-    <col min="7" max="7" width="27.42578125" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" customWidth="1"/>
-    <col min="10" max="10" width="36.5703125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" customWidth="1"/>
+    <col min="3" max="3" width="41.5" customWidth="1"/>
+    <col min="4" max="4" width="45.1640625" customWidth="1"/>
+    <col min="5" max="5" width="40.6640625" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="27.5" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.5" customWidth="1"/>
+    <col min="10" max="10" width="36.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="12" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="17" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="7">
         <f ca="1">NOW()</f>
-        <v>45977.76065960648</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="27" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
+        <v>45992.756913194447</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="28" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-    </row>
-    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+    </row>
+    <row r="6" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1053,7 +1506,7 @@
       <c r="G6" t="s">
         <v>33</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="1" t="s">
         <v>34</v>
       </c>
       <c r="I6" t="s">
@@ -1063,17 +1516,65 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="8"/>
+    <row r="7" spans="1:10" ht="106" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="4"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="4"/>
+    </row>
+    <row r="8" spans="1:10" ht="61" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="4"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1081,6 +1582,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D2" location="'Severity &amp; Priority Key'!A1" display="Select to view the Severity &amp; Priority Rating Key " xr:uid="{F3949ABE-C1BE-4FE3-8718-03631FA7FAA9}"/>
+    <hyperlink ref="D3" location="'TC Naming Convention'!A1" display="Select to view the Test Case Naming Convention Guildelines" xr:uid="{10D22FC2-51FB-E942-B611-1B6C2F5ABE52}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1092,33 +1594,33 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{983C971C-B98C-4FF5-90C7-7BD846EDF5A8}">
   <dimension ref="A2:E18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" customWidth="1"/>
-    <col min="2" max="2" width="41.7109375" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" customWidth="1"/>
-    <col min="5" max="5" width="41.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41.6640625" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="41.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="4" spans="1:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="4" spans="1:5" ht="22" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="D4" s="3" t="s">
+      <c r="B4" s="15"/>
+      <c r="D4" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E4" s="16"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1132,77 +1634,77 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>23</v>
       </c>
@@ -1222,4 +1724,181 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF5B3B75-26ED-484A-8B59-1ACD1F246C4F}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="28" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="34"/>
+    </row>
+    <row r="2" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="31"/>
+      <c r="H2" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="49"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="43"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="43"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="41" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="43"/>
+    </row>
+    <row r="6" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="46"/>
+    </row>
+    <row r="7" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+    </row>
+    <row r="8" spans="1:11" ht="22" x14ac:dyDescent="0.2">
+      <c r="A8" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="22"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="25"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="36"/>
+      <c r="I10" s="37"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="28"/>
+    </row>
+    <row r="12" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="40"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="18"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H2:K2" location="'Test Cases'!A1" display="BRING ME BACK TO THE TEST CASES!" xr:uid="{911CF568-580C-164D-A5BF-770889D8D684}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>